<commit_message>
update ups data 2026-09-15 14:08
</commit_message>
<xml_diff>
--- a/ups_prev.xlsx
+++ b/ups_prev.xlsx
@@ -42263,7 +42263,7 @@
       </c>
       <c r="F1136" t="inlineStr">
         <is>
-          <t>قيد العمل - المهندس</t>
+          <t>استكمال التعديلات</t>
         </is>
       </c>
       <c r="G1136" t="inlineStr">
@@ -46736,7 +46736,7 @@
       </c>
       <c r="F1257" t="inlineStr">
         <is>
-          <t>قيد العمل - المهندس</t>
+          <t>قيد العمل - مشرف رخص البناء</t>
         </is>
       </c>
       <c r="G1257" t="inlineStr">
@@ -47661,7 +47661,7 @@
       </c>
       <c r="F1282" t="inlineStr">
         <is>
-          <t>قيد العمل - المهندس</t>
+          <t>قيد العمل - مشرف رخص البناء</t>
         </is>
       </c>
       <c r="G1282" t="inlineStr">
@@ -48031,7 +48031,7 @@
       </c>
       <c r="F1292" t="inlineStr">
         <is>
-          <t>بانتظار السداد</t>
+          <t>مكتمل</t>
         </is>
       </c>
       <c r="G1292" t="inlineStr">
@@ -49844,7 +49844,7 @@
       </c>
       <c r="F1341" t="inlineStr">
         <is>
-          <t>بانتظار السداد</t>
+          <t>مكتمل</t>
         </is>
       </c>
       <c r="G1341" t="inlineStr">
@@ -51398,7 +51398,7 @@
       </c>
       <c r="F1383" t="inlineStr">
         <is>
-          <t>بانتظار السداد</t>
+          <t>مكتمل</t>
         </is>
       </c>
       <c r="G1383" t="inlineStr">
@@ -51649,7 +51649,7 @@
       </c>
       <c r="F1390" t="inlineStr">
         <is>
-          <t>قيد العمل - المهندس</t>
+          <t>استكمال التعديلات</t>
         </is>
       </c>
       <c r="G1390" t="inlineStr">
@@ -52204,7 +52204,7 @@
       </c>
       <c r="F1405" t="inlineStr">
         <is>
-          <t>قيد العمل - المهندس</t>
+          <t>استكمال التعديلات</t>
         </is>
       </c>
       <c r="G1405" t="inlineStr">

</xml_diff>